<commit_message>
webapp: visualizador de presupuesto (2 escenarios, baja el costo a la mitad) + torre de giro con ingeniería real
- Visualizador de costos (botón 💰 Costos): tarjetas Máximo vs Económico
  ($612.000 → $282.000 CLP, −54%), barras por subsistema y tabla de "cómo bajar
  cada ítem". Descarga Excel/CSV. Deep-link #cost. Datos en docs/costos.json.
- Remodelado del mecanismo como RODAMIENTO DE GIRO CENTRAL (slewing ring) con
  DOS caminos de carga separados: el peso del usuario baja por un pedestal central
  fijo (por el bore del rodamiento) a la placa base; el rodamiento solo toma el
  giro y el momento del brazo. Apilado real abajo→arriba: placa base + patas ·
  pista fija + bolas + pista giratoria · brazo/carro · pedestal · plataforma arriba.
- Panel derecho: la observación "POR REVISAR" pasa a nota de ingeniería resuelta.
- Nuevos query params para compartir/capturar estados: ?explode ?cam ?tgt

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/costos-antofagasta-clp.xlsx
+++ b/docs/costos-antofagasta-clp.xlsx
@@ -111,9 +111,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -485,28 +483,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OpenOmni — Costo maximo estimado (Antofagasta, Chile)</t>
+          <t>OpenOmni - Costos (Antofagasta, Chile) - CLP</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Pesos chilenos (CLP). Precios de referencia tope; edita cantidades/precios y los totales se recalculan.</t>
+          <t>Escenario MAXIMO vs ECONOMICO (rescatando/sustituyendo). Edita cant/precios y recalcula.</t>
         </is>
       </c>
     </row>
@@ -528,17 +528,27 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Precio unit. (CLP)</t>
+          <t>Precio max</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Subtotal (CLP)</t>
+          <t>Subtotal max</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Notas / donde</t>
+          <t>Precio ECO</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Subtotal ECO</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Como bajar de precio</t>
         </is>
       </c>
     </row>
@@ -565,16 +575,23 @@
         <f>C6*D6</f>
         <v/>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Sodimac / Construmart</t>
+      <c r="F6" s="6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G6" s="6">
+        <f>C6*F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>OSB / pallet reciclado</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Pino 2x4" (3.2m) - vigas radiales</t>
+          <t>Pino 2x4" radiales</t>
         </is>
       </c>
       <c r="C7" s="5" t="n">
@@ -587,16 +604,23 @@
         <f>C7*D7</f>
         <v/>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>estructura tipo rayos</t>
+      <c r="F7" s="6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G7" s="6">
+        <f>C7*F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>pallet / rescatado</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Pino 2x12" - bloque central octagono</t>
+          <t>Pino 2x12" bloque central</t>
         </is>
       </c>
       <c r="C8" s="5" t="n">
@@ -609,12 +633,23 @@
         <f>C8*D8</f>
         <v/>
       </c>
-      <c r="F8" s="5" t="inlineStr"/>
+      <c r="F8" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G8" s="6">
+        <f>C8*F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>madera rescatada</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Tornillos estructurales 8x80mm (caja)</t>
+          <t>Tornillos estructurales 8x80mm</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
@@ -627,16 +662,23 @@
         <f>C9*D9</f>
         <v/>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>juntas radial-centro</t>
+      <c r="F9" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G9" s="6">
+        <f>C9*F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>menos cantidad</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Tornillos madera 4x40mm (caja 200)</t>
+          <t>Tornillos madera 4x40mm</t>
         </is>
       </c>
       <c r="C10" s="5" t="n">
@@ -649,16 +691,19 @@
         <f>C10*D10</f>
         <v/>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>deck a radiales</t>
-        </is>
-      </c>
+      <c r="F10" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G10" s="6">
+        <f>C10*F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Adhesivo maderas D3 (250ml)</t>
+          <t>Adhesivo maderas D3</t>
         </is>
       </c>
       <c r="C11" s="5" t="n">
@@ -671,12 +716,19 @@
         <f>C11*D11</f>
         <v/>
       </c>
-      <c r="F11" s="5" t="inlineStr"/>
+      <c r="F11" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G11" s="6">
+        <f>C11*F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Lamina HDPE / melamina lisa (superficie)</t>
+          <t>Superficie deslizante</t>
         </is>
       </c>
       <c r="C12" s="5" t="n">
@@ -689,9 +741,16 @@
         <f>C12*D12</f>
         <v/>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>cara deslizante</t>
+      <c r="F12" s="6" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G12" s="6">
+        <f>C12*F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>alfombra + deslizadores (DIY) en vez de HDPE</t>
         </is>
       </c>
     </row>
@@ -711,14 +770,17 @@
         <f>C13*D13</f>
         <v/>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>baja friccion</t>
-        </is>
-      </c>
+      <c r="F13" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G13" s="6">
+        <f>C13*F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="D14" s="7" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
@@ -727,18 +789,22 @@
         <f>SUM(E6:E13)</f>
         <v/>
       </c>
+      <c r="G14" s="8">
+        <f>SUM(G6:G13)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Giro (anillo turntable) + fierros</t>
+          <t>Giro (anillo/collar) + fierros</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Rodamiento plato giratorio / lazy-susan grande</t>
+          <t>Rodamiento giratorio del collar</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
@@ -751,16 +817,23 @@
         <f>C17*D17</f>
         <v/>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>el collar giratorio</t>
+      <c r="F17" s="6" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G17" s="6">
+        <f>C17*F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>lazy-susan barato / rueda auto rescatada</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Ruedas / rodillos industriales (respaldo)</t>
+          <t>Ruedas / rodillos</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
@@ -773,12 +846,23 @@
         <f>C18*D18</f>
         <v/>
       </c>
-      <c r="F18" s="5" t="inlineStr"/>
+      <c r="F18" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G18" s="6">
+        <f>C18*F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>rescatadas</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Tubo cuadrado acero 40x40x3mm (6m)</t>
+          <t>Tubo cuadrado 40x40x3mm (6m)</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
@@ -791,16 +875,23 @@
         <f>C19*D19</f>
         <v/>
       </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>eslabon inferior brazo</t>
+      <c r="F19" s="6" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G19" s="6">
+        <f>C19*F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>fierro usado</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Tubo cuadrado acero 50x50x3mm (2m)</t>
+          <t>Tubo cuadrado 50x50x3mm (2m)</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
@@ -813,16 +904,23 @@
         <f>C20*D20</f>
         <v/>
       </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>poste</t>
+      <c r="F20" s="6" t="n">
+        <v>7000</v>
+      </c>
+      <c r="G20" s="6">
+        <f>C20*F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>fierro usado</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Rodamientos 6008 (juntas del brazo)</t>
+          <t>Rodamientos 6008 (juntas)</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
@@ -835,12 +933,23 @@
         <f>C21*D21</f>
         <v/>
       </c>
-      <c r="F21" s="5" t="inlineStr"/>
+      <c r="F21" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G21" s="6">
+        <f>C21*F21</f>
+        <v/>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>de bicicleta rescatados</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Pernos M10/M12 grado 8.8 + tuercas</t>
+          <t>Pernos M10/M12 8.8 + tuercas</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
@@ -853,11 +962,14 @@
         <f>C22*D22</f>
         <v/>
       </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>ejes / doble corte</t>
-        </is>
-      </c>
+      <c r="F22" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G22" s="6">
+        <f>C22*F22</f>
+        <v/>
+      </c>
+      <c r="H22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="B23" s="5" t="inlineStr">
@@ -875,16 +987,19 @@
         <f>C23*D23</f>
         <v/>
       </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>junta del codo</t>
-        </is>
-      </c>
+      <c r="F23" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G23" s="6">
+        <f>C23*F23</f>
+        <v/>
+      </c>
+      <c r="H23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Cierre rapido (QR) de bicicleta</t>
+          <t>Cierre rapido (QR) bici</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
@@ -897,14 +1012,21 @@
         <f>C24*D24</f>
         <v/>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>bloqueo del brazo</t>
+      <c r="F24" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G24" s="6">
+        <f>C24*F24</f>
+        <v/>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>rescatado</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="D25" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
@@ -913,6 +1035,10 @@
         <f>SUM(E17:E24)</f>
         <v/>
       </c>
+      <c r="G25" s="8">
+        <f>SUM(G17:G24)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -924,7 +1050,7 @@
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Resorte a gas 300-400N, carrera &gt;=120mm</t>
+          <t>Resorte a gas 300-400N</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
@@ -937,9 +1063,16 @@
         <f>C28*D28</f>
         <v/>
       </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>o cilindro silla oficina</t>
+      <c r="F28" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G28" s="6">
+        <f>C28*F28</f>
+        <v/>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>cilindro de silla de oficina rescatado</t>
         </is>
       </c>
     </row>
@@ -959,14 +1092,17 @@
         <f>C29*D29</f>
         <v/>
       </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>montaje del strut</t>
-        </is>
-      </c>
+      <c r="F29" s="6" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G29" s="6">
+        <f>C29*F29</f>
+        <v/>
+      </c>
+      <c r="H29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="D30" s="7" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
@@ -975,6 +1111,10 @@
         <f>SUM(E28:E29)</f>
         <v/>
       </c>
+      <c r="G30" s="8">
+        <f>SUM(G28:G29)</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -986,7 +1126,7 @@
     <row r="33">
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Cinturon lumbar / arnes acolchado</t>
+          <t>Cinturon lumbar / arnes</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
@@ -999,16 +1139,23 @@
         <f>C33*D33</f>
         <v/>
       </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>interfaz cuerpo-brazo</t>
+      <c r="F33" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G33" s="6">
+        <f>C33*F33</f>
+        <v/>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>arnes que ya tengas</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Deslizadores PTFE/UHMW (muebles)</t>
+          <t>Deslizadores PTFE/UHMW</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
@@ -1021,9 +1168,16 @@
         <f>C34*D34</f>
         <v/>
       </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>almohadillas del calzado</t>
+      <c r="F34" s="6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G34" s="6">
+        <f>C34*F34</f>
+        <v/>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>deslizadores de muebles basicos</t>
         </is>
       </c>
     </row>
@@ -1043,12 +1197,19 @@
         <f>C35*D35</f>
         <v/>
       </c>
-      <c r="F35" s="5" t="inlineStr"/>
+      <c r="F35" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G35" s="6">
+        <f>C35*F35</f>
+        <v/>
+      </c>
+      <c r="H35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Filamento PETG 1kg (piezas impresas)</t>
+          <t>Filamento PETG 1kg</t>
         </is>
       </c>
       <c r="C36" s="5" t="n">
@@ -1061,10 +1222,21 @@
         <f>C36*D36</f>
         <v/>
       </c>
-      <c r="F36" s="5" t="inlineStr"/>
+      <c r="F36" s="6" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G36" s="6">
+        <f>C36*F36</f>
+        <v/>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>PLA / menos filamento</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="D37" s="7" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
@@ -1073,6 +1245,10 @@
         <f>SUM(E33:E36)</f>
         <v/>
       </c>
+      <c r="G37" s="8">
+        <f>SUM(G33:G36)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -1084,7 +1260,7 @@
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>ESP32-C3 (tracker de pie)</t>
+          <t>ESP32-C3 (tracker)</t>
         </is>
       </c>
       <c r="C40" s="5" t="n">
@@ -1097,16 +1273,23 @@
         <f>C40*D40</f>
         <v/>
       </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>AliExpress / local</t>
+      <c r="F40" s="6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G40" s="6">
+        <f>C40*F40</f>
+        <v/>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>ESP32 generico</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>IMU MPU-9250 / ICM-20948</t>
+          <t>IMU MPU-9250</t>
         </is>
       </c>
       <c r="C41" s="5" t="n">
@@ -1119,12 +1302,23 @@
         <f>C41*D41</f>
         <v/>
       </c>
-      <c r="F41" s="5" t="inlineStr"/>
+      <c r="F41" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G41" s="6">
+        <f>C41*F41</f>
+        <v/>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>MPU6050 (6 ejes)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>FSR sensor de fuerza (talon)</t>
+          <t>FSR sensor de fuerza</t>
         </is>
       </c>
       <c r="C42" s="5" t="n">
@@ -1137,12 +1331,23 @@
         <f>C42*D42</f>
         <v/>
       </c>
-      <c r="F42" s="5" t="inlineStr"/>
+      <c r="F42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="6">
+        <f>C42*F42</f>
+        <v/>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>omitir: deteccion solo por IMU</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>LiPo 500-1000mAh + cargador TP4056</t>
+          <t>LiPo + TP4056</t>
         </is>
       </c>
       <c r="C43" s="5" t="n">
@@ -1155,12 +1360,19 @@
         <f>C43*D43</f>
         <v/>
       </c>
-      <c r="F43" s="5" t="inlineStr"/>
+      <c r="F43" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G43" s="6">
+        <f>C43*F43</f>
+        <v/>
+      </c>
+      <c r="H43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>ESP32-S3 (hub = mando USB)</t>
+          <t>ESP32-S3 (hub)</t>
         </is>
       </c>
       <c r="C44" s="5" t="n">
@@ -1173,12 +1385,19 @@
         <f>C44*D44</f>
         <v/>
       </c>
-      <c r="F44" s="5" t="inlineStr"/>
+      <c r="F44" s="6" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G44" s="6">
+        <f>C44*F44</f>
+        <v/>
+      </c>
+      <c r="H44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Cables, JST, headers, resistencias</t>
+          <t>Cables, JST, headers</t>
         </is>
       </c>
       <c r="C45" s="5" t="n">
@@ -1191,10 +1410,17 @@
         <f>C45*D45</f>
         <v/>
       </c>
-      <c r="F45" s="5" t="inlineStr"/>
+      <c r="F45" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G45" s="6">
+        <f>C45*F45</f>
+        <v/>
+      </c>
+      <c r="H45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="D46" s="7" t="inlineStr">
+      <c r="C46" s="7" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
@@ -1203,6 +1429,10 @@
         <f>SUM(E40:E45)</f>
         <v/>
       </c>
+      <c r="G46" s="8">
+        <f>SUM(G40:G45)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -1227,16 +1457,19 @@
         <f>C49*D49</f>
         <v/>
       </c>
-      <c r="F49" s="5" t="inlineStr">
-        <is>
-          <t>acabado del cuenco</t>
-        </is>
-      </c>
+      <c r="F49" s="6" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G49" s="6">
+        <f>C49*F49</f>
+        <v/>
+      </c>
+      <c r="H49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Grasa para rodamientos</t>
+          <t>Grasa rodamientos</t>
         </is>
       </c>
       <c r="C50" s="5" t="n">
@@ -1249,7 +1482,14 @@
         <f>C50*D50</f>
         <v/>
       </c>
-      <c r="F50" s="5" t="inlineStr"/>
+      <c r="F50" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G50" s="6">
+        <f>C50*F50</f>
+        <v/>
+      </c>
+      <c r="H50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="B51" s="5" t="inlineStr">
@@ -1267,14 +1507,21 @@
         <f>C51*D51</f>
         <v/>
       </c>
-      <c r="F51" s="5" t="inlineStr">
-        <is>
-          <t>colchon</t>
+      <c r="F51" s="6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G51" s="6">
+        <f>C51*F51</f>
+        <v/>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>menos colchon</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="D52" s="7" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
@@ -1283,28 +1530,38 @@
         <f>SUM(E49:E51)</f>
         <v/>
       </c>
+      <c r="G52" s="8">
+        <f>SUM(G49:G51)</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
-      <c r="D54" s="9" t="inlineStr">
-        <is>
-          <t>TOTAL MAXIMO</t>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="E54" s="10">
         <f>E14+E25+E30+E37+E46+E52</f>
         <v/>
       </c>
+      <c r="G54" s="10">
+        <f>G14+G25+G30+G37+G46+G52</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A48:F48"/>
-    <mergeCell ref="A39:F39"/>
+  <mergeCells count="10">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A27:H27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>